<commit_message>
feat(interviews): import historique lit le type d'entretien par ligne
Ajoute la colonne "Type Entretien" à l'import CSV d'historique
d'entretiens pour permettre de mélanger plusieurs types dans un même
fichier ; le type choisi dans l'interface devient une valeur par
défaut appliquée quand la colonne est vide.
</commit_message>
<xml_diff>
--- a/doc/Exemple Importation/template_entretiens_historique.xlsx
+++ b/doc/Exemple Importation/template_entretiens_historique.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D999"/>
+  <dimension ref="A1:E999"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -428,26 +428,31 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Matricule</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>État</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Date prévue</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Date de réalisation</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Type Entretien</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>

</xml_diff>